<commit_message>
docs: add Master Settings list (workbook + guide) for super-admin settings
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CentralLists_Import.xlsx
+++ b/docs/CentralLists_Import.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Model Specs" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Activity Log" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Hub Items" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Master Settings" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -272,6 +273,19 @@
     <tableColumn id="4" name="Item Id"/>
     <tableColumn id="5" name="Payload"/>
     <tableColumn id="6" name="Rev"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="T_MasterSettings" displayName="T_MasterSettings" ref="A1:D2" headerRowCount="1">
+  <autoFilter ref="A1:D2"/>
+  <tableColumns count="4">
+    <tableColumn id="1" name="Title"/>
+    <tableColumn id="2" name="Value"/>
+    <tableColumn id="3" name="Secret"/>
+    <tableColumn id="4" name="Description"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -566,7 +580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -584,7 +598,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Site: https://nucor.sharepoint.com/sites/bg.ter.O365.TERALIT</t>
+          <t>Site: NBG Hub Data (dedicated site)</t>
         </is>
       </c>
     </row>
@@ -787,6 +801,23 @@
       <c r="C23" s="5" t="inlineStr">
         <is>
           <t>Title = division:kind:id. Delete the example row after import. Change Payload to Multiple lines of text (plain). Leave Rev as text. Then index Division and Kind.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Master Settings</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Inventory - Master Settings</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Delete the example row after import. Change Value to Multiple lines of text (plain). Then set UNIQUE PERMISSIONS (see MANUAL_LIST_SETUP.md): everyone Read, Owners only Edit.</t>
         </is>
       </c>
     </row>
@@ -1523,4 +1554,71 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>EXAMPLE-DELETE</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>example-value</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Title = setting key (for example lenovo_client_id or super_admins)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>